<commit_message>
Update registration database and Excel/CSV submissions dataset
</commit_message>
<xml_diff>
--- a/data/submissions.xlsx
+++ b/data/submissions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,26 +480,26 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arun Kumar V</t>
+          <t>ABHIJIT V 2025-2029</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>22AM099</t>
+          <t>SEC25AM112</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>arun.v@sairam.edu.in</t>
+          <t>sec25am112@sairamtap.edu.in</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+91 94441 22334</t>
+          <t>98405649063</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -509,57 +509,49 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3rd Year</t>
+          <t>2nd Year</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Natural Language Processing</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://github.com/arun-nlp</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Excited to build reasoning agents and local LLM pipelines.</t>
-        </is>
-      </c>
+          <t>Computer Vision &amp; Generative AI</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-07 17:23:58</t>
+          <t>2026-09-07 23:23:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rithanya Shree</t>
+          <t>Arun Kumar V</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22AM105</t>
+          <t>22AM099</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>rithanya.s@sairam.edu.in</t>
+          <t>arun.v@sairam.edu.in</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+91 99401 88776</t>
+          <t>+91 94441 22334</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -569,22 +561,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2nd Year</t>
+          <t>3rd Year</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Computer Vision &amp; Generative AI</t>
+          <t>Natural Language Processing</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://github.com/rithanya-vision</t>
+          <t>https://github.com/arun-nlp</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Excited to train generative diffusion models in CCIC!</t>
+          <t>Excited to build reasoning agents and local LLM pipelines.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -594,32 +586,32 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-09-07 17:23:23</t>
+          <t>2026-09-07 17:23:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Test Registration Student</t>
+          <t>Rithanya Shree</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23AM999</t>
+          <t>22AM105</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>test.student@sairam.edu.in</t>
+          <t>rithanya.s@sairam.edu.in</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+91 99999 88888</t>
+          <t>+91 99401 88776</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -639,12 +631,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://github.com/test</t>
+          <t>https://github.com/rithanya-vision</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Excited to build models in CCIC!</t>
+          <t>Excited to train generative diffusion models in CCIC!</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -654,32 +646,32 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-09-07 17:22:39</t>
+          <t>2026-09-07 17:23:23</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Harish Kumar</t>
+          <t>Test Registration Student</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>22AM099</t>
+          <t>23AM999</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>harish.k@sairam.edu.in</t>
+          <t>test.student@sairam.edu.in</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+91 98409 11223</t>
+          <t>+91 99999 88888</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -689,38 +681,38 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3rd Year</t>
+          <t>2nd Year</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Natural Language Processing</t>
+          <t>Computer Vision &amp; Generative AI</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://github.com/harish-nlp</t>
+          <t>https://github.com/test</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Excited to work with LLM architectures and automated reasoning agents in CCIC.</t>
+          <t>Excited to build models in CCIC!</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-09-07 16:32:31</t>
+          <t>2026-09-07 17:22:39</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -774,122 +766,122 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-09-07 16:31:50</t>
+          <t>2026-09-07 16:32:31</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rahul Varman</t>
+          <t>Harish Kumar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>22IT033</t>
+          <t>22AM099</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>rahul.v@sairam.edu.in</t>
+          <t>harish.k@sairam.edu.in</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>+91 98412 67890</t>
+          <t>+91 98409 11223</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CSE (AI &amp; ML)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2nd Year</t>
+          <t>3rd Year</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Edge AI &amp; IoT Systems</t>
+          <t>Natural Language Processing</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>linkedin.com/in/rahulvarman</t>
+          <t>https://github.com/harish-nlp</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Developing low-latency TinyML applications for industrial edge sensors.</t>
+          <t>Excited to work with LLM architectures and automated reasoning agents in CCIC.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-09-07 16:28:52</t>
+          <t>2026-09-07 16:31:50</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sneha Ramesh</t>
+          <t>Rahul Varman</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23AM078</t>
+          <t>22IT033</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>sneha.r@sairam.edu.in</t>
+          <t>rahul.v@sairam.edu.in</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>+91 98841 54321</t>
+          <t>+91 98412 67890</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CSE (AI &amp; ML)</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1st Year</t>
+          <t>2nd Year</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; Data Science</t>
+          <t>Edge AI &amp; IoT Systems</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>github.com/sneha-codes</t>
+          <t>linkedin.com/in/rahulvarman</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Enthusiastic beginner in ML eager to learn and participate in national hackathons.</t>
+          <t>Developing low-latency TinyML applications for industrial edge sensors.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Reviewed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -900,56 +892,56 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Karthik Raja</t>
+          <t>Sneha Ramesh</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>21CS089</t>
+          <t>23AM078</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>karthik.r@sairam.edu.in</t>
+          <t>sneha.r@sairam.edu.in</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>+91 94440 98765</t>
+          <t>+91 98841 54321</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CSE (AI &amp; ML)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3rd Year</t>
+          <t>1st Year</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Deep Reinforcement Learning &amp; Robotics</t>
+          <t>Machine Learning &amp; Data Science</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>github.com/karthik-robolab</t>
+          <t>github.com/sneha-codes</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Building autonomous robotics algorithms and edge AI controllers.</t>
+          <t>Enthusiastic beginner in ML eager to learn and participate in national hackathons.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Reviewed</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -960,56 +952,56 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Divya Krishnan</t>
+          <t>Karthik Raja</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>22AM045</t>
+          <t>21CS089</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>divya.k@sairam.edu.in</t>
+          <t>karthik.r@sairam.edu.in</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>+91 97102 34567</t>
+          <t>+91 94440 98765</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CSE (AI &amp; ML)</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2nd Year</t>
+          <t>3rd Year</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Natural Language Processing</t>
+          <t>Deep Reinforcement Learning &amp; Robotics</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>linkedin.com/in/divyakrishnan</t>
+          <t>github.com/karthik-robolab</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Eager to contribute to CCIC NLP research labs and open-source LLM agents.</t>
+          <t>Building autonomous robotics algorithms and edge AI controllers.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1020,59 +1012,119 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Divya Krishnan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>22AM045</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>divya.k@sairam.edu.in</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>+91 97102 34567</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>CSE (AI &amp; ML)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2nd Year</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/divyakrishnan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Eager to contribute to CCIC NLP research labs and open-source LLM agents.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-07 16:28:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
         <v>1</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Aravind Swaminathan</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>21AM012</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>aravind.s@sairam.edu.in</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>+91 98401 23456</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>CSE (AI &amp; ML)</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>3rd Year</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Computer Vision &amp; Generative AI</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>github.com/aravind-ai</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Passionate about building state-of-the-art vision models for healthcare diagnosis.</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-09-07 16:28:52</t>
         </is>

</xml_diff>